<commit_message>
Move Final column position
</commit_message>
<xml_diff>
--- a/leaderboard.xlsx
+++ b/leaderboard.xlsx
@@ -453,32 +453,32 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Round 1</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Round 2</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Round 3</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Round 4</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Round 5</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Final</t>
         </is>
       </c>
     </row>
@@ -498,22 +498,22 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>97.33</v>
+        <v>896.33</v>
       </c>
       <c r="F2" t="n">
         <v>97.33</v>
       </c>
       <c r="G2" t="n">
+        <v>97.33</v>
+      </c>
+      <c r="H2" t="n">
         <v>96.33</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>92.67</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>77</v>
-      </c>
-      <c r="J2" t="n">
-        <v>896.33</v>
       </c>
     </row>
     <row r="3">
@@ -532,22 +532,22 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
+        <v>892.67</v>
+      </c>
+      <c r="F3" t="n">
         <v>96</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>96.33</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>94.67</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>84</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>32.33</v>
-      </c>
-      <c r="J3" t="n">
-        <v>892.67</v>
       </c>
     </row>
     <row r="4">
@@ -566,22 +566,22 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
+        <v>882</v>
+      </c>
+      <c r="F4" t="n">
         <v>92.67</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>96.67</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>92.33</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>84.33</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>1.67</v>
-      </c>
-      <c r="J4" t="n">
-        <v>882</v>
       </c>
     </row>
     <row r="5">
@@ -600,22 +600,22 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
+        <v>866.33</v>
+      </c>
+      <c r="F5" t="n">
         <v>94.67</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>87.33</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>91.67</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>84</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>53.33</v>
-      </c>
-      <c r="J5" t="n">
-        <v>866.33</v>
       </c>
     </row>
     <row r="6">
@@ -634,22 +634,22 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
+        <v>859.33</v>
+      </c>
+      <c r="F6" t="n">
         <v>93.67</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>97</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>94.33</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>85.67</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>46.67</v>
-      </c>
-      <c r="J6" t="n">
-        <v>859.33</v>
       </c>
     </row>
     <row r="7">
@@ -668,22 +668,22 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
+        <v>834.67</v>
+      </c>
+      <c r="F7" t="n">
         <v>95.67</v>
-      </c>
-      <c r="F7" t="n">
-        <v>96</v>
       </c>
       <c r="G7" t="n">
         <v>96</v>
       </c>
       <c r="H7" t="n">
+        <v>96</v>
+      </c>
+      <c r="I7" t="n">
         <v>84.67</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>59</v>
-      </c>
-      <c r="J7" t="n">
-        <v>834.67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>